<commit_message>
SLO: sequence column (asal kitab ki tarteeb)
</commit_message>
<xml_diff>
--- a/static/slo_import_template.xlsx
+++ b/static/slo_import_template.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SLO" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -415,15 +415,6 @@
   </sheetPr>
   <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -458,7 +449,7 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>book_pages</t>
+          <t>sequence</t>
         </is>
       </c>
     </row>
@@ -489,10 +480,8 @@
           <t>Pre-writing</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>4-5</t>
-        </is>
+      <c r="G2" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -522,10 +511,8 @@
           <t>Number</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>12-14</t>
-        </is>
+      <c r="G3" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="4">
@@ -555,10 +542,8 @@
           <t>Comparison</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>22</t>
-        </is>
+      <c r="G4" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="5">
@@ -588,10 +573,8 @@
           <t>Flat Shape</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>30-31</t>
-        </is>
+      <c r="G5" t="n">
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>